<commit_message>
feat: merge VK contacts for allowlisted parties, add missing candidates
- only process rows of the 5 allowed parties
- fill/append ВКонтакте from VK 1 and VK 2, no duplicates
- unwrap broken HYPERLINK cells to real URLs
- append missing candidates as new rows (Мотрюков, Тольяттинский округ)
- regenerate site
</commit_message>
<xml_diff>
--- a/candidates.xlsx
+++ b/candidates.xlsx
@@ -8,9 +8,7 @@
   <sheets>
     <sheet name="Кандидаты по округам" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Кандидаты по округам'!$A$1:$F$1611</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -409,7 +407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1611"/>
+  <dimension ref="A1:M1612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.28515625" customWidth="1" min="1" max="1"/>
@@ -722,7 +720,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://vk.com/club230166777; https://vk.com/shudraldpr</t>
+          <t>https://vk.com/club230166777;  https://vk.com/shudraldpr; https://vk.com/shudraldpr</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1605,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://vk.com/julia.zhdanova29</t>
+          <t>https://vk.com/julia.zhdanova29; https://vk.ru/zhdanova_29</t>
         </is>
       </c>
     </row>
@@ -2002,7 +2000,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>vk.com/mashaborh; https://vk.com/mashaborh</t>
+          <t>vk.com/mashaborh;  https://vk.com/mashaborh; https://vk.com/mashaborh</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2250,6 +2248,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sevostyanov39</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2317,7 +2320,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://HYPERLINK is not implemented. linkLocation=https://vk.com/id642668509</t>
+          <t>https://vk.com/id642668509</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2420,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>vk.com/ngrumyantsev; https://vk.com/ngrumyantsev</t>
+          <t>vk.com/ngrumyantsev;  https://vk.com/ngrumyantsev; https://vk.com/ngrumyantsev</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2910,6 +2913,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id528435876</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3007,7 +3015,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://vk.com/id1108898505</t>
+          <t>https://vk.com/id1108898505; https://vk.ru/olegmatytsin</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3105,6 +3113,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tmk1395</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3307,7 +3320,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://HYPERLINK is not implemented. linkLocation=https://vk.com/id53559048</t>
+          <t>https://vk.com/id53559048</t>
         </is>
       </c>
     </row>
@@ -3750,6 +3763,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://vk.ru/nikpnik</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4070,6 +4088,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kravitrock</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4590,6 +4613,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>https://vk.ru/irina_mozalevskaya</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -4982,7 +5010,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>http://vk.com/anponomarev; https://vk.com/anponomarev</t>
+          <t>http://vk.com/anponomarev;  https://vk.com/anponomarev; https://vk.com/anponomarev</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -5150,6 +5178,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kovalenko_dmitriy71</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -5260,6 +5293,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id71974592</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -5465,6 +5503,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>https://vk.ru/anodon</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -5565,6 +5608,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id259826467</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -5597,7 +5645,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>https://HYPERLINK is not implemented. linkLocation=https://vk.com/id49131842</t>
+          <t>https://vk.com/id49131842; https://vk.ru/artur1503</t>
         </is>
       </c>
     </row>
@@ -5730,6 +5778,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>https://vk.ru/a.dorofeev.dnrsovet</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -5795,6 +5848,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1106507607</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -5827,7 +5885,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>https://HYPERLINK is not implemented. linkLocation=https://vk.com/public237221197</t>
+          <t>https://vk.com/public237221197; https://vk.ru/seleznevgk</t>
         </is>
       </c>
     </row>
@@ -5962,7 +6020,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>https://HYPERLINK is not implemented. linkLocation=https://vk.com/id707763012</t>
+          <t>https://vk.com/id707763012</t>
         </is>
       </c>
     </row>
@@ -6040,6 +6098,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id274513111</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -6190,6 +6253,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tatianaslutskaiia</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -6970,6 +7038,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id384512908</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -7330,6 +7403,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>https://vk.ru/new_leed</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -7360,6 +7438,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>https://vk.ru/komandalogunova</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -8355,6 +8438,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>https://vk.ru/l.yuditsky</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -8682,7 +8770,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>http://vk.com/marinaorgeeva; https://vk.com/marinaorgeeva</t>
+          <t>http://vk.com/marinaorgeeva;  https://vk.com/marinaorgeeva; https://vk.com/marinaorgeeva</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -8855,6 +8943,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aleshkin5s</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -9645,6 +9738,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>https://vk.com/id33608806</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -9677,7 +9775,7 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>https://vk.com/antongorelkin; https://vk.com/gorelkin.official</t>
+          <t>https://vk.com/antongorelkin;  https://vk.com/gorelkin.official; https://vk.com/gorelkin.official</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
@@ -9887,7 +9985,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>http://vk.com/petrov_parlament; https://vk.com/petrov_parlament</t>
+          <t>http://vk.com/petrov_parlament;  https://vk.com/petrov_parlament; https://vk.com/petrov_parlament</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -10245,6 +10343,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://vk.ru/medved_resto</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -10652,7 +10755,7 @@
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>https://vk.com/olgatyrykina</t>
+          <t>https://vk.com/olgatyrykina; https://vk.ru/o.tyrykina</t>
         </is>
       </c>
     </row>
@@ -10880,6 +10983,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>https://vk.ru/krospecialolympics</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -11007,7 +11115,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>https://vk.com/club236132544</t>
+          <t>https://vk.com/club236132544; https://vk.ru/id716569547</t>
         </is>
       </c>
     </row>
@@ -11440,6 +11548,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>https://vk.com/i.shibalkin</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -11530,6 +11643,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>https://vk.ru/questltd</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -11700,6 +11818,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>https://vk.ru/nikolyapu13</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -11910,6 +12033,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>https://vk.ru/valery_doc_ldpr</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -12005,6 +12133,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>https://vk.ru/v.pronkin76</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -12502,7 +12635,7 @@
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>https://vk.com/club237224250; https://vk.com/priemnaya_ezubov</t>
+          <t>https://vk.com/club237224250;  https://vk.com/priemnaya_ezubov; https://vk.com/priemnaya_ezubov</t>
         </is>
       </c>
       <c r="H363" t="inlineStr">
@@ -12962,7 +13095,7 @@
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>https://vk.com/maxim_zolotyhin</t>
+          <t>https://vk.com/maxim_zolotyhin; https://vk.ru/zolotuhin_maxim</t>
         </is>
       </c>
     </row>
@@ -13250,6 +13383,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id866661877</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -13310,6 +13448,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://vk.ru/senderskysemyon</t>
+        </is>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="n">
@@ -13340,6 +13483,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://vk.ru/martyinuk; https://vk.ru/id178593009</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -13450,6 +13598,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://vk.ru/isaev_valery</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="n">
@@ -13690,6 +13843,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://vk.ru/semizorovpavel</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="n">
@@ -13750,6 +13908,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dvdubrov</t>
+        </is>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="n">
@@ -14325,6 +14488,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://vk.ru/konstantintimopheev</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
@@ -14387,7 +14555,7 @@
       </c>
       <c r="G421" t="inlineStr">
         <is>
-          <t>http://vk.com/vasiliipiskarev; https://vk.com/vasiliipiskarev</t>
+          <t>http://vk.com/vasiliipiskarev;  https://vk.com/vasiliipiskarev; https://vk.com/vasiliipiskarev</t>
         </is>
       </c>
       <c r="H421" t="inlineStr">
@@ -14525,6 +14693,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://vk.ru/mitrofanova11</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="n">
@@ -14925,6 +15098,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://vk.ru/svsadriev</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="n">
@@ -15185,6 +15363,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vkatorgina</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="n">
@@ -16260,6 +16443,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>https://vk.ru/zinoviev_sergei</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" t="n">
@@ -16657,7 +16845,7 @@
       </c>
       <c r="G489" t="inlineStr">
         <is>
-          <t>https://vk.ru/va_gusev; https://vk.com/va_gusev</t>
+          <t>https://vk.ru/va_gusev;  https://vk.com/va_gusev; https://vk.com/va_gusev</t>
         </is>
       </c>
       <c r="H489" t="inlineStr">
@@ -16852,7 +17040,7 @@
       </c>
       <c r="G494" t="inlineStr">
         <is>
-          <t>https://vk.ru/popovrtr; https://vk.com/popovrtr</t>
+          <t>https://vk.ru/popovrtr;  https://vk.com/popovrtr; https://vk.com/popovrtr</t>
         </is>
       </c>
       <c r="H494" t="inlineStr">
@@ -17840,6 +18028,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>https://vk.ru/latyntsevalexander</t>
+        </is>
+      </c>
     </row>
     <row r="521">
       <c r="A521" t="n">
@@ -23725,6 +23918,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>https://vk.ru/samsonov_sp</t>
+        </is>
+      </c>
     </row>
     <row r="684">
       <c r="A684" t="n">
@@ -23755,6 +23953,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tumanov6sotok</t>
+        </is>
+      </c>
     </row>
     <row r="685">
       <c r="A685" t="n">
@@ -23915,6 +24118,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>https://vk.ru/deputatsp1979</t>
+        </is>
+      </c>
     </row>
     <row r="690">
       <c r="A690" t="n">
@@ -24290,6 +24498,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id159019876</t>
+        </is>
+      </c>
     </row>
     <row r="701">
       <c r="A701" t="n">
@@ -24380,6 +24593,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>https://vk.ru/bulgakov__aa</t>
+        </is>
+      </c>
     </row>
     <row r="704">
       <c r="A704" t="n">
@@ -24410,6 +24628,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id286704121</t>
+        </is>
+      </c>
     </row>
     <row r="705">
       <c r="A705" t="n">
@@ -24647,7 +24870,7 @@
       </c>
       <c r="G711" t="inlineStr">
         <is>
-          <t>https://vk.com/vatalinyv?ysclid=ly60fean1v846862277</t>
+          <t>https://vk.com/vatalinyv?ysclid=ly60fean1v846862277; https://vk.com/vatalinyv</t>
         </is>
       </c>
     </row>
@@ -24682,7 +24905,7 @@
       </c>
       <c r="G712" t="inlineStr">
         <is>
-          <t>https://vk.com/stanislavgontar?from=search</t>
+          <t>https://vk.com/stanislavgontar?from=search; https://vk.com/stanislavgontar</t>
         </is>
       </c>
       <c r="L712" t="inlineStr">
@@ -24755,6 +24978,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id108910392</t>
+        </is>
+      </c>
     </row>
     <row r="715">
       <c r="A715" t="n">
@@ -25185,6 +25413,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>https://vk.ru/annatatarinzeva</t>
+        </is>
+      </c>
     </row>
     <row r="728">
       <c r="A728" t="n">
@@ -25470,6 +25703,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id12979508</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="n">
@@ -25760,6 +25998,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>https://vk.ru/yulya_garevskaya</t>
+        </is>
+      </c>
     </row>
     <row r="746">
       <c r="A746" t="n">
@@ -25890,6 +26133,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id140622720</t>
+        </is>
+      </c>
     </row>
     <row r="750">
       <c r="A750" t="n">
@@ -26190,6 +26438,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>https://vk.ru/il.prihodko; https://vk.ru/novoemestovn</t>
+        </is>
+      </c>
     </row>
     <row r="759">
       <c r="A759" t="n">
@@ -26545,6 +26798,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>https://vk.ru/radkevich_alexey</t>
+        </is>
+      </c>
     </row>
     <row r="770">
       <c r="A770" t="n">
@@ -27235,6 +27493,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id442573938</t>
+        </is>
+      </c>
     </row>
     <row r="791">
       <c r="A791" t="n">
@@ -27770,6 +28033,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>https://vk.ru/maxim_makalenko</t>
+        </is>
+      </c>
     </row>
     <row r="807">
       <c r="A807" t="n">
@@ -27992,7 +28260,7 @@
       </c>
       <c r="G813" t="inlineStr">
         <is>
-          <t>https://vk.com/deputat_smolin; https://vk.com/smolinomsk</t>
+          <t>https://vk.com/deputat_smolin;  https://vk.com/smolinomsk; https://vk.com/smolinomsk</t>
         </is>
       </c>
       <c r="J813" t="inlineStr">
@@ -28275,6 +28543,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>https://vk.ru/rodionov.maxim</t>
+        </is>
+      </c>
     </row>
     <row r="822">
       <c r="A822" t="n">
@@ -29045,6 +29318,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>https://vk.ru/idynkovich; https://vk.ru/i.dynkovich</t>
+        </is>
+      </c>
     </row>
     <row r="845">
       <c r="A845" t="n">
@@ -29500,6 +29778,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vasilev5800</t>
+        </is>
+      </c>
     </row>
     <row r="858">
       <c r="A858" t="n">
@@ -29702,7 +29985,7 @@
       </c>
       <c r="G863" t="inlineStr">
         <is>
-          <t>http://vk.com/igorrudensky; https://vk.com/igorrudensky</t>
+          <t>http://vk.com/igorrudensky;  https://vk.com/igorrudensky; https://vk.com/igorrudensky</t>
         </is>
       </c>
       <c r="H863" t="inlineStr">
@@ -30582,7 +30865,7 @@
       </c>
       <c r="G889" t="inlineStr">
         <is>
-          <t>https://vk.com/postnikov.ldpr/</t>
+          <t>https://vk.com/postnikov.ldpr/; https://vk.com/postnikov.ldpr</t>
         </is>
       </c>
       <c r="H889" t="inlineStr">
@@ -31210,6 +31493,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>https://vk.ru/darkpsionik</t>
+        </is>
+      </c>
     </row>
     <row r="909">
       <c r="A909" t="n">
@@ -31240,6 +31528,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vasyutkin</t>
+        </is>
+      </c>
     </row>
     <row r="910">
       <c r="A910" t="n">
@@ -32045,6 +32338,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id249295027</t>
+        </is>
+      </c>
     </row>
     <row r="935">
       <c r="A935" t="n">
@@ -32435,6 +32733,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>https://vk.ru/azat_vachitovich</t>
+        </is>
+      </c>
     </row>
     <row r="947">
       <c r="A947" t="n">
@@ -32755,6 +33058,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sukharevdpr</t>
+        </is>
+      </c>
     </row>
     <row r="957">
       <c r="A957" t="n">
@@ -33025,6 +33333,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id6032193</t>
+        </is>
+      </c>
     </row>
     <row r="965">
       <c r="A965" t="n">
@@ -33615,6 +33928,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>https://vk.ru/zavadichpv</t>
+        </is>
+      </c>
     </row>
     <row r="983">
       <c r="A983" t="n">
@@ -33930,6 +34248,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>https://vk.ru/muratpayzulaev</t>
+        </is>
+      </c>
     </row>
     <row r="993">
       <c r="A993" t="n">
@@ -33960,6 +34283,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dzhavatxanov</t>
+        </is>
+      </c>
     </row>
     <row r="994">
       <c r="A994" t="n">
@@ -34020,6 +34348,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>https://vk.ru/daniyal_gadzhiev</t>
+        </is>
+      </c>
     </row>
     <row r="996">
       <c r="A996" t="n">
@@ -34050,6 +34383,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>https://vk.ru/mr.gazilaev</t>
+        </is>
+      </c>
     </row>
     <row r="997">
       <c r="A997" t="n">
@@ -34140,6 +34478,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>https://vk.ru/nurbagandov_nm</t>
+        </is>
+      </c>
       <c r="H999" t="inlineStr">
         <is>
           <t>https://t.me/s/nurbagandov_nm</t>
@@ -34180,6 +34523,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id490059117</t>
+        </is>
+      </c>
     </row>
     <row r="1001">
       <c r="A1001" t="n">
@@ -34270,6 +34618,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id594418467</t>
+        </is>
+      </c>
     </row>
     <row r="1004">
       <c r="A1004" t="n">
@@ -34460,6 +34813,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1009" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id526416848</t>
+        </is>
+      </c>
     </row>
     <row r="1010">
       <c r="A1010" t="n">
@@ -34530,6 +34888,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id740944111</t>
+        </is>
+      </c>
     </row>
     <row r="1012">
       <c r="A1012" t="n">
@@ -34620,6 +34983,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id770173996</t>
+        </is>
+      </c>
     </row>
     <row r="1015">
       <c r="A1015" t="n">
@@ -34680,6 +35048,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id798073784</t>
+        </is>
+      </c>
     </row>
     <row r="1017">
       <c r="A1017" t="n">
@@ -34710,6 +35083,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1017" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id63549232</t>
+        </is>
+      </c>
     </row>
     <row r="1018">
       <c r="A1018" t="n">
@@ -34740,6 +35118,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1018" t="inlineStr">
+        <is>
+          <t>https://vk.ru/migmir64</t>
+        </is>
+      </c>
     </row>
     <row r="1019">
       <c r="A1019" t="n">
@@ -34890,6 +35273,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1023" t="inlineStr">
+        <is>
+          <t>https://vk.ru/izyumov_royne</t>
+        </is>
+      </c>
     </row>
     <row r="1024">
       <c r="A1024" t="n">
@@ -35045,6 +35433,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1028" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id100368398</t>
+        </is>
+      </c>
     </row>
     <row r="1029">
       <c r="A1029" t="n">
@@ -35075,6 +35468,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1029" t="inlineStr">
+        <is>
+          <t>https://vk.ru/a.i.monastyrshin</t>
+        </is>
+      </c>
     </row>
     <row r="1030">
       <c r="A1030" t="n">
@@ -35135,6 +35533,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1031" t="inlineStr">
+        <is>
+          <t>https://vk.com/saladina_tatiana</t>
+        </is>
+      </c>
     </row>
     <row r="1032">
       <c r="A1032" t="n">
@@ -35165,6 +35568,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1032" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id36440914</t>
+        </is>
+      </c>
     </row>
     <row r="1033">
       <c r="A1033" t="n">
@@ -35225,6 +35633,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1034" t="inlineStr">
+        <is>
+          <t>https://vk.ru/s.kochev11</t>
+        </is>
+      </c>
     </row>
     <row r="1035">
       <c r="A1035" t="n">
@@ -35322,7 +35735,7 @@
       </c>
       <c r="G1037" t="inlineStr">
         <is>
-          <t>https://vk.com/mihajlovoleg; https://vk.com/mikkomi</t>
+          <t>https://vk.com/mihajlovoleg;  https://vk.com/mikkomi; https://vk.com/mikkomi</t>
         </is>
       </c>
     </row>
@@ -35355,6 +35768,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id166024764</t>
+        </is>
+      </c>
     </row>
     <row r="1039">
       <c r="A1039" t="n">
@@ -35475,6 +35893,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1042" t="inlineStr">
+        <is>
+          <t>https://vk.ru/gv_kovalenko</t>
+        </is>
+      </c>
     </row>
     <row r="1043">
       <c r="A1043" t="n">
@@ -35605,6 +36028,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1046" t="inlineStr">
+        <is>
+          <t>https://vk.ru/yanina.pavlenko</t>
+        </is>
+      </c>
     </row>
     <row r="1047">
       <c r="A1047" t="n">
@@ -35995,6 +36423,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1058" t="inlineStr">
+        <is>
+          <t>https://vk.ru/n.popov77</t>
+        </is>
+      </c>
     </row>
     <row r="1059">
       <c r="A1059" t="n">
@@ -36195,6 +36628,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1064" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id138861501</t>
+        </is>
+      </c>
     </row>
     <row r="1065">
       <c r="A1065" t="n">
@@ -36510,6 +36948,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>https://vk.com/id440822915</t>
+        </is>
+      </c>
     </row>
     <row r="1075">
       <c r="A1075" t="n">
@@ -36605,6 +37048,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id6126967</t>
+        </is>
+      </c>
     </row>
     <row r="1078">
       <c r="A1078" t="n">
@@ -36800,6 +37248,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id326656214</t>
+        </is>
+      </c>
       <c r="H1083" t="inlineStr">
         <is>
           <t>https://t.me/parahingp</t>
@@ -36835,6 +37288,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id198404863</t>
+        </is>
+      </c>
     </row>
     <row r="1085">
       <c r="A1085" t="n">
@@ -37060,6 +37518,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>https://vk.ru/svbestaev</t>
+        </is>
+      </c>
     </row>
     <row r="1092">
       <c r="A1092" t="n">
@@ -37090,6 +37553,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>https://vk.ru/chermendudaev</t>
+        </is>
+      </c>
     </row>
     <row r="1093">
       <c r="A1093" t="n">
@@ -37210,6 +37678,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id496825121</t>
+        </is>
+      </c>
     </row>
     <row r="1097">
       <c r="A1097" t="n">
@@ -37280,6 +37753,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id19950500</t>
+        </is>
+      </c>
     </row>
     <row r="1099">
       <c r="A1099" t="n">
@@ -37310,6 +37788,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1099" t="inlineStr">
+        <is>
+          <t>https://vk.ru/delta_cf</t>
+        </is>
+      </c>
     </row>
     <row r="1100">
       <c r="A1100" t="n">
@@ -37370,6 +37853,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1101" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id790933399</t>
+        </is>
+      </c>
     </row>
     <row r="1102">
       <c r="A1102" t="n">
@@ -37435,6 +37923,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id5819308</t>
+        </is>
+      </c>
     </row>
     <row r="1104">
       <c r="A1104" t="n">
@@ -37525,6 +38018,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1106" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id162944736</t>
+        </is>
+      </c>
     </row>
     <row r="1107">
       <c r="A1107" t="n">
@@ -37765,6 +38263,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1113" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id96020299</t>
+        </is>
+      </c>
     </row>
     <row r="1114">
       <c r="A1114" t="n">
@@ -37825,6 +38328,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1115" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id537295047</t>
+        </is>
+      </c>
     </row>
     <row r="1116">
       <c r="A1116" t="n">
@@ -37885,6 +38393,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sudykinsergey</t>
+        </is>
+      </c>
     </row>
     <row r="1118">
       <c r="A1118" t="n">
@@ -37915,6 +38428,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vakhitov9090</t>
+        </is>
+      </c>
     </row>
     <row r="1119">
       <c r="A1119" t="n">
@@ -38005,6 +38523,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>https://vk.ru/k.evseev_116</t>
+        </is>
+      </c>
     </row>
     <row r="1122">
       <c r="A1122" t="n">
@@ -38170,6 +38693,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>https://vk.com/artyw</t>
+        </is>
+      </c>
     </row>
     <row r="1127">
       <c r="A1127" t="n">
@@ -38200,6 +38728,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>https://vk.ru/syaldyshev</t>
+        </is>
+      </c>
     </row>
     <row r="1128">
       <c r="A1128" t="n">
@@ -38260,6 +38793,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id259133372</t>
+        </is>
+      </c>
     </row>
     <row r="1130">
       <c r="A1130" t="n">
@@ -38290,6 +38828,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id720877868</t>
+        </is>
+      </c>
     </row>
     <row r="1131">
       <c r="A1131" t="n">
@@ -38320,6 +38863,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id29617919</t>
+        </is>
+      </c>
     </row>
     <row r="1132">
       <c r="A1132" t="n">
@@ -38390,6 +38938,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>https://vk.ru/starostinvn</t>
+        </is>
+      </c>
     </row>
     <row r="1134">
       <c r="A1134" t="n">
@@ -38420,6 +38973,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id639769941</t>
+        </is>
+      </c>
     </row>
     <row r="1135">
       <c r="A1135" t="n">
@@ -38540,6 +39098,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tarassinonyan</t>
+        </is>
+      </c>
     </row>
     <row r="1139">
       <c r="A1139" t="n">
@@ -38660,6 +39223,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sizyakin</t>
+        </is>
+      </c>
     </row>
     <row r="1143">
       <c r="A1143" t="n">
@@ -38690,6 +39258,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id826066660</t>
+        </is>
+      </c>
     </row>
     <row r="1144">
       <c r="A1144" t="n">
@@ -38720,6 +39293,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>https://vk.ru/i.b.simakov</t>
+        </is>
+      </c>
     </row>
     <row r="1145">
       <c r="A1145" t="n">
@@ -38750,6 +39328,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>https://vk.ru/rozhkov_sergey</t>
+        </is>
+      </c>
     </row>
     <row r="1146">
       <c r="A1146" t="n">
@@ -38810,6 +39393,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dedovich_kommunist</t>
+        </is>
+      </c>
     </row>
     <row r="1148">
       <c r="A1148" t="n">
@@ -38840,6 +39428,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>https://vk.ru/mvchumakov</t>
+        </is>
+      </c>
     </row>
     <row r="1149">
       <c r="A1149" t="n">
@@ -38990,6 +39583,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>https://vk.ru/medvedev_sovetnik</t>
+        </is>
+      </c>
     </row>
     <row r="1154">
       <c r="A1154" t="n">
@@ -39020,6 +39618,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>https://vk.ru/rumyantsevaldpr</t>
+        </is>
+      </c>
     </row>
     <row r="1155">
       <c r="A1155" t="n">
@@ -39050,6 +39653,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>https://vk.ru/germanza</t>
+        </is>
+      </c>
     </row>
     <row r="1156">
       <c r="A1156" t="n">
@@ -39082,7 +39690,7 @@
       </c>
       <c r="G1156" t="inlineStr">
         <is>
-          <t>http://vk.com/evgeny_bessonov; https://vk.com/evgeny_bessonov</t>
+          <t>http://vk.com/evgeny_bessonov;  https://vk.com/evgeny_bessonov; https://vk.com/evgeny_bessonov</t>
         </is>
       </c>
     </row>
@@ -39145,6 +39753,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vitaly_miroshnikov</t>
+        </is>
+      </c>
     </row>
     <row r="1159">
       <c r="A1159" t="n">
@@ -39210,6 +39823,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>https://vk.ru/pavlenko178</t>
+        </is>
+      </c>
     </row>
     <row r="1161">
       <c r="A1161" t="n">
@@ -39240,6 +39858,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>https://vk.ru/idvelichkoartem</t>
+        </is>
+      </c>
     </row>
     <row r="1162">
       <c r="A1162" t="n">
@@ -39270,6 +39893,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id804876003</t>
+        </is>
+      </c>
     </row>
     <row r="1163">
       <c r="A1163" t="n">
@@ -39300,6 +39928,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id595213071</t>
+        </is>
+      </c>
     </row>
     <row r="1164">
       <c r="A1164" t="n">
@@ -39330,6 +39963,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ilinovmaksim</t>
+        </is>
+      </c>
     </row>
     <row r="1165">
       <c r="A1165" t="n">
@@ -39360,6 +39998,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id649997669</t>
+        </is>
+      </c>
     </row>
     <row r="1166">
       <c r="A1166" t="n">
@@ -39420,6 +40063,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id4399080</t>
+        </is>
+      </c>
     </row>
     <row r="1168">
       <c r="A1168" t="n">
@@ -39480,6 +40128,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>https://vk.ru/abakumov1973</t>
+        </is>
+      </c>
     </row>
     <row r="1170">
       <c r="A1170" t="n">
@@ -39510,6 +40163,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aleksei.misan</t>
+        </is>
+      </c>
     </row>
     <row r="1171">
       <c r="A1171" t="n">
@@ -39650,6 +40308,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tbguscova</t>
+        </is>
+      </c>
     </row>
     <row r="1175">
       <c r="A1175" t="n">
@@ -39745,6 +40408,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id135038789</t>
+        </is>
+      </c>
     </row>
     <row r="1178">
       <c r="A1178" t="n">
@@ -39775,6 +40443,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ldprpavelrzn</t>
+        </is>
+      </c>
     </row>
     <row r="1179">
       <c r="A1179" t="n">
@@ -39807,7 +40480,7 @@
       </c>
       <c r="G1179" t="inlineStr">
         <is>
-          <t>https://vk.com/krasovandrey</t>
+          <t>https://vk.com/krasovandrey; https://vk.com/krasovandreypublic</t>
         </is>
       </c>
       <c r="H1179" t="inlineStr">
@@ -39875,6 +40548,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ivanfrommurmansk</t>
+        </is>
+      </c>
     </row>
     <row r="1182">
       <c r="A1182" t="n">
@@ -39905,6 +40583,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>https://vk.ru/norkrzn</t>
+        </is>
+      </c>
     </row>
     <row r="1183">
       <c r="A1183" t="n">
@@ -39965,6 +40648,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1184" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1107038551</t>
+        </is>
+      </c>
     </row>
     <row r="1185">
       <c r="A1185" t="n">
@@ -39995,6 +40683,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1185" t="inlineStr">
+        <is>
+          <t>https://vk.ru/morozov_evgeny_rzn</t>
+        </is>
+      </c>
     </row>
     <row r="1186">
       <c r="A1186" t="n">
@@ -40025,6 +40718,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1186" t="inlineStr">
+        <is>
+          <t>https://vk.ru/depytatmystafin; https://vk.ru/maksimmystafinldpr</t>
+        </is>
+      </c>
     </row>
     <row r="1187">
       <c r="A1187" t="n">
@@ -40055,6 +40753,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1187" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tomchuk_people; https://vk.ru/tomchuk_as</t>
+        </is>
+      </c>
     </row>
     <row r="1188">
       <c r="A1188" t="n">
@@ -40310,6 +41013,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1195" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sanyadeputat</t>
+        </is>
+      </c>
     </row>
     <row r="1196">
       <c r="A1196" t="n">
@@ -40340,6 +41048,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1196" t="inlineStr">
+        <is>
+          <t>https://vk.ru/mikhailmarykhin</t>
+        </is>
+      </c>
     </row>
     <row r="1197">
       <c r="A1197" t="n">
@@ -40430,6 +41143,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1199" t="inlineStr">
+        <is>
+          <t>https://vk.ru/oleg_sakeev</t>
+        </is>
+      </c>
     </row>
     <row r="1200">
       <c r="A1200" t="n">
@@ -40525,6 +41243,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1202" t="inlineStr">
+        <is>
+          <t>https://vk.ru/markarow</t>
+        </is>
+      </c>
     </row>
     <row r="1203">
       <c r="A1203" t="n">
@@ -40555,6 +41278,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1203" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id341814431</t>
+        </is>
+      </c>
     </row>
     <row r="1204">
       <c r="A1204" t="n">
@@ -40585,6 +41313,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1204" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id166866042</t>
+        </is>
+      </c>
     </row>
     <row r="1205">
       <c r="A1205" t="n">
@@ -40615,6 +41348,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dportnyagin161</t>
+        </is>
+      </c>
     </row>
     <row r="1206">
       <c r="A1206" t="n">
@@ -40717,7 +41455,7 @@
       </c>
       <c r="G1208" t="inlineStr">
         <is>
-          <t>https://m.vk.com/id811543193; https://vk.ru/id811543193</t>
+          <t>https://m.vk.com/id811543193;  https://vk.ru/id811543193; https://vk.ru/id811543193</t>
         </is>
       </c>
       <c r="H1208" t="inlineStr">
@@ -40755,6 +41493,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>https://vk.ru/mguseynov</t>
+        </is>
+      </c>
     </row>
     <row r="1210">
       <c r="A1210" t="n">
@@ -40905,6 +41648,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>https://vk.ru/yulia.pletneva</t>
+        </is>
+      </c>
     </row>
     <row r="1215">
       <c r="A1215" t="n">
@@ -40935,6 +41683,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>https://vk.ru/alex_zhivaikin</t>
+        </is>
+      </c>
     </row>
     <row r="1216">
       <c r="A1216" t="n">
@@ -41000,6 +41753,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>https://vk.ru/maksim_venediktov</t>
+        </is>
+      </c>
     </row>
     <row r="1218">
       <c r="A1218" t="n">
@@ -41030,6 +41788,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id2389826</t>
+        </is>
+      </c>
     </row>
     <row r="1219">
       <c r="A1219" t="n">
@@ -41060,6 +41823,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>https://vk.ru/milyaev</t>
+        </is>
+      </c>
     </row>
     <row r="1220">
       <c r="A1220" t="n">
@@ -41090,6 +41858,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>https://vk.com/deputatlozhechko</t>
+        </is>
+      </c>
     </row>
     <row r="1221">
       <c r="A1221" t="n">
@@ -41180,6 +41953,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sazoncev</t>
+        </is>
+      </c>
     </row>
     <row r="1224">
       <c r="A1224" t="n">
@@ -41210,6 +41988,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>https://vk.ru/svetlanajazzpolice</t>
+        </is>
+      </c>
     </row>
     <row r="1225">
       <c r="A1225" t="n">
@@ -41240,6 +42023,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id162568759</t>
+        </is>
+      </c>
     </row>
     <row r="1226">
       <c r="A1226" t="n">
@@ -41340,6 +42128,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>https://vk.ru/lelik190</t>
+        </is>
+      </c>
     </row>
     <row r="1229">
       <c r="A1229" t="n">
@@ -41475,6 +42268,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1232" t="inlineStr">
+        <is>
+          <t>https://vk.ru/zverev_aa</t>
+        </is>
+      </c>
     </row>
     <row r="1233">
       <c r="A1233" t="n">
@@ -41505,6 +42303,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1233" t="inlineStr">
+        <is>
+          <t>https://vk.ru/priemnayaivanova</t>
+        </is>
+      </c>
     </row>
     <row r="1234">
       <c r="A1234" t="n">
@@ -41535,6 +42338,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1234" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vbelikov_zaks</t>
+        </is>
+      </c>
     </row>
     <row r="1235">
       <c r="A1235" t="n">
@@ -41595,6 +42403,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1236" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id422742618; https://vk.ru/vladimirmatyagin</t>
+        </is>
+      </c>
     </row>
     <row r="1237">
       <c r="A1237" t="n">
@@ -41655,6 +42468,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1238" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id598404242</t>
+        </is>
+      </c>
     </row>
     <row r="1239">
       <c r="A1239" t="n">
@@ -41715,6 +42533,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1240" t="inlineStr">
+        <is>
+          <t>https://vk.ru/mamashanatasha</t>
+        </is>
+      </c>
     </row>
     <row r="1241">
       <c r="A1241" t="n">
@@ -41805,6 +42628,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1243" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id65745235</t>
+        </is>
+      </c>
     </row>
     <row r="1244">
       <c r="A1244" t="n">
@@ -41835,6 +42663,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1244" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tatarovalery</t>
+        </is>
+      </c>
     </row>
     <row r="1245">
       <c r="A1245" t="n">
@@ -41895,6 +42728,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1246" t="inlineStr">
+        <is>
+          <t>https://vk.ru/pykhteevas</t>
+        </is>
+      </c>
     </row>
     <row r="1247">
       <c r="A1247" t="n">
@@ -42140,6 +42978,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1254" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1125730888</t>
+        </is>
+      </c>
     </row>
     <row r="1255">
       <c r="A1255" t="n">
@@ -42200,6 +43043,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1256" t="inlineStr">
+        <is>
+          <t>https://vk.ru/club240805995</t>
+        </is>
+      </c>
     </row>
     <row r="1257">
       <c r="A1257" t="n">
@@ -42230,6 +43078,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1257" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id794727226; https://vk.ru/prokopenko_k</t>
+        </is>
+      </c>
     </row>
     <row r="1258">
       <c r="A1258" t="n">
@@ -42260,6 +43113,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1258" t="inlineStr">
+        <is>
+          <t>https://vk.ru/egormixailov_kprf</t>
+        </is>
+      </c>
     </row>
     <row r="1259">
       <c r="A1259" t="n">
@@ -42290,6 +43148,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1259" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id642866969</t>
+        </is>
+      </c>
       <c r="H1259" t="inlineStr">
         <is>
           <t>https://t.me/oxdmitrieva</t>
@@ -42390,6 +43253,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1262" t="inlineStr">
+        <is>
+          <t>https://vk.ru/marinalebedeva1959</t>
+        </is>
+      </c>
     </row>
     <row r="1263">
       <c r="A1263" t="n">
@@ -42450,6 +43318,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1264" t="inlineStr">
+        <is>
+          <t>https://vk.ru/egorova_deputat</t>
+        </is>
+      </c>
     </row>
     <row r="1265">
       <c r="A1265" t="n">
@@ -42480,6 +43353,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1265" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id4183010</t>
+        </is>
+      </c>
     </row>
     <row r="1266">
       <c r="A1266" t="n">
@@ -42510,6 +43388,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1266" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1360928</t>
+        </is>
+      </c>
     </row>
     <row r="1267">
       <c r="A1267" t="n">
@@ -42570,6 +43453,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1268" t="inlineStr">
+        <is>
+          <t>https://vk.ru/malkov2026</t>
+        </is>
+      </c>
     </row>
     <row r="1269">
       <c r="A1269" t="n">
@@ -42670,6 +43558,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1271" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ivliev_sn</t>
+        </is>
+      </c>
     </row>
     <row r="1272">
       <c r="A1272" t="n">
@@ -42760,6 +43653,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1274" t="inlineStr">
+        <is>
+          <t>https://vk.ru/revinaa</t>
+        </is>
+      </c>
     </row>
     <row r="1275">
       <c r="A1275" t="n">
@@ -42850,6 +43748,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1277" t="inlineStr">
+        <is>
+          <t>https://vk.ru/volodin.saratov</t>
+        </is>
+      </c>
       <c r="H1277" t="inlineStr">
         <is>
           <t>https://t.me/vv_volodin</t>
@@ -42890,6 +43793,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1278" t="inlineStr">
+        <is>
+          <t>https://vk.ru/denisanb</t>
+        </is>
+      </c>
     </row>
     <row r="1279">
       <c r="A1279" t="n">
@@ -42985,6 +43893,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1281" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id35792092</t>
+        </is>
+      </c>
     </row>
     <row r="1282">
       <c r="A1282" t="n">
@@ -43075,6 +43988,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1284" t="inlineStr">
+        <is>
+          <t>https://vk.ru/antonina.galyashkina</t>
+        </is>
+      </c>
     </row>
     <row r="1285">
       <c r="A1285" t="n">
@@ -43137,7 +44055,7 @@
       </c>
       <c r="G1286" t="inlineStr">
         <is>
-          <t>https://vk.com/aleksandranidalov?ysclid=l4wsi1m9l130981001</t>
+          <t>https://vk.com/aleksandranidalov?ysclid=l4wsi1m9l130981001; https://vk.com/aleksandranidalov</t>
         </is>
       </c>
     </row>
@@ -43200,6 +44118,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>https://vk.ru/evgeuk</t>
+        </is>
+      </c>
     </row>
     <row r="1289">
       <c r="A1289" t="n">
@@ -43420,6 +44343,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id364512772</t>
+        </is>
+      </c>
     </row>
     <row r="1296">
       <c r="A1296" t="n">
@@ -43480,6 +44408,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id907478</t>
+        </is>
+      </c>
     </row>
     <row r="1298">
       <c r="A1298" t="n">
@@ -43770,6 +44703,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id808225161</t>
+        </is>
+      </c>
     </row>
     <row r="1307">
       <c r="A1307" t="n">
@@ -43832,7 +44770,7 @@
       </c>
       <c r="G1308" t="inlineStr">
         <is>
-          <t>https://vk.com/karlovga</t>
+          <t>https://vk.com/karlovga; https://vk.com/g.a.karlov</t>
         </is>
       </c>
       <c r="H1308" t="inlineStr">
@@ -43910,6 +44848,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ashikhmin_kprf</t>
+        </is>
+      </c>
       <c r="H1310" t="inlineStr">
         <is>
           <t>https://t.me/ashikhmin_deputat65</t>
@@ -44135,6 +45078,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id137033638</t>
+        </is>
+      </c>
     </row>
     <row r="1317">
       <c r="A1317" t="n">
@@ -44165,6 +45113,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>https://vk.ru/evgnkolo</t>
+        </is>
+      </c>
     </row>
     <row r="1318">
       <c r="A1318" t="n">
@@ -44195,6 +45148,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>https://vk.ru/lyubov_kuntsevich</t>
+        </is>
+      </c>
     </row>
     <row r="1319">
       <c r="A1319" t="n">
@@ -44295,6 +45253,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id18810026</t>
+        </is>
+      </c>
     </row>
     <row r="1322">
       <c r="A1322" t="n">
@@ -44475,6 +45438,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>https://vk.ru/v_smirnov96</t>
+        </is>
+      </c>
     </row>
     <row r="1328">
       <c r="A1328" t="n">
@@ -44505,6 +45473,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id462826737</t>
+        </is>
+      </c>
     </row>
     <row r="1329">
       <c r="A1329" t="n">
@@ -44565,6 +45538,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sergey_kozin_sr</t>
+        </is>
+      </c>
     </row>
     <row r="1331">
       <c r="A1331" t="n">
@@ -44595,6 +45573,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dymshakov</t>
+        </is>
+      </c>
     </row>
     <row r="1332">
       <c r="A1332" t="n">
@@ -44625,6 +45608,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id358712771</t>
+        </is>
+      </c>
     </row>
     <row r="1333">
       <c r="A1333" t="n">
@@ -44655,6 +45643,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id162340028</t>
+        </is>
+      </c>
     </row>
     <row r="1334">
       <c r="A1334" t="n">
@@ -44685,6 +45678,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aleksey_svalov</t>
+        </is>
+      </c>
     </row>
     <row r="1335">
       <c r="A1335" t="n">
@@ -44780,6 +45778,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>https://vk.ru/es.popov</t>
+        </is>
+      </c>
     </row>
     <row r="1338">
       <c r="A1338" t="n">
@@ -44840,6 +45843,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id857764884</t>
+        </is>
+      </c>
     </row>
     <row r="1340">
       <c r="A1340" t="n">
@@ -44870,6 +45878,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>https://vk.ru/n.musalnikova</t>
+        </is>
+      </c>
     </row>
     <row r="1341">
       <c r="A1341" t="n">
@@ -44930,6 +45943,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vinogradova121</t>
+        </is>
+      </c>
     </row>
     <row r="1343">
       <c r="A1343" t="n">
@@ -44990,6 +46008,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>https://vk.ru/z.zhuravleva</t>
+        </is>
+      </c>
     </row>
     <row r="1345">
       <c r="A1345" t="n">
@@ -45020,6 +46043,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id468187701</t>
+        </is>
+      </c>
     </row>
     <row r="1346">
       <c r="A1346" t="n">
@@ -45115,6 +46143,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1348" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id63073797</t>
+        </is>
+      </c>
     </row>
     <row r="1349">
       <c r="A1349" t="n">
@@ -45175,6 +46208,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1350" t="inlineStr">
+        <is>
+          <t>https://vk.ru/alexdigi</t>
+        </is>
+      </c>
     </row>
     <row r="1351">
       <c r="A1351" t="n">
@@ -45345,6 +46383,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1355" t="inlineStr">
+        <is>
+          <t>https://vk.ru/burgart_za</t>
+        </is>
+      </c>
     </row>
     <row r="1356">
       <c r="A1356" t="n">
@@ -45420,6 +46463,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1357" t="inlineStr">
+        <is>
+          <t>https://vk.ru/realbarybin</t>
+        </is>
+      </c>
     </row>
     <row r="1358">
       <c r="A1358" t="n">
@@ -45450,6 +46498,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>https://vk.ru/brakovenkova</t>
+        </is>
+      </c>
     </row>
     <row r="1359">
       <c r="A1359" t="n">
@@ -45510,6 +46563,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1360" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tyoma090580</t>
+        </is>
+      </c>
     </row>
     <row r="1361">
       <c r="A1361" t="n">
@@ -45580,6 +46638,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1362" t="inlineStr">
+        <is>
+          <t>https://vk.ru/shotput</t>
+        </is>
+      </c>
     </row>
     <row r="1363">
       <c r="A1363" t="n">
@@ -45700,6 +46763,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1366" t="inlineStr">
+        <is>
+          <t>https://vk.ru/emelyanovkprf</t>
+        </is>
+      </c>
     </row>
     <row r="1367">
       <c r="A1367" t="n">
@@ -45820,6 +46888,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1370" t="inlineStr">
+        <is>
+          <t>https://vk.ru/staskireev_ru</t>
+        </is>
+      </c>
     </row>
     <row r="1371">
       <c r="A1371" t="n">
@@ -45915,6 +46988,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kazakovaolga_rf</t>
+        </is>
+      </c>
       <c r="H1373" t="inlineStr">
         <is>
           <t>https://t.me/s/kazakovaolga_rf</t>
@@ -46075,6 +47153,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>https://vk.ru/solodovaap</t>
+        </is>
+      </c>
     </row>
     <row r="1379">
       <c r="A1379" t="n">
@@ -46225,6 +47308,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aiserdykov777</t>
+        </is>
+      </c>
     </row>
     <row r="1384">
       <c r="A1384" t="n">
@@ -46435,6 +47523,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id557272955</t>
+        </is>
+      </c>
     </row>
     <row r="1391">
       <c r="A1391" t="n">
@@ -46465,6 +47558,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id197530697</t>
+        </is>
+      </c>
     </row>
     <row r="1392">
       <c r="A1392" t="n">
@@ -46600,6 +47698,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1395" t="inlineStr">
+        <is>
+          <t>https://vk.ru/lozovoy1960</t>
+        </is>
+      </c>
     </row>
     <row r="1396">
       <c r="A1396" t="n">
@@ -46765,6 +47868,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1400" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id4886983</t>
+        </is>
+      </c>
     </row>
     <row r="1401">
       <c r="A1401" t="n">
@@ -46795,6 +47903,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1401" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id357148029</t>
+        </is>
+      </c>
     </row>
     <row r="1402">
       <c r="A1402" t="n">
@@ -46855,6 +47968,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1403" t="inlineStr">
+        <is>
+          <t>https://vk.ru/levshukovdn</t>
+        </is>
+      </c>
     </row>
     <row r="1404">
       <c r="A1404" t="n">
@@ -46885,6 +48003,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1404" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id283014989</t>
+        </is>
+      </c>
     </row>
     <row r="1405">
       <c r="A1405" t="n">
@@ -46945,6 +48068,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1406" t="inlineStr">
+        <is>
+          <t>https://vk.ru/karpovtver</t>
+        </is>
+      </c>
     </row>
     <row r="1407">
       <c r="A1407" t="n">
@@ -47135,6 +48263,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1412" t="inlineStr">
+        <is>
+          <t>https://vk.ru/englushkova</t>
+        </is>
+      </c>
     </row>
     <row r="1413">
       <c r="A1413" t="n">
@@ -47195,6 +48328,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1414" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id178782683</t>
+        </is>
+      </c>
     </row>
     <row r="1415">
       <c r="A1415" t="n">
@@ -47350,6 +48488,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1418" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1033192307</t>
+        </is>
+      </c>
     </row>
     <row r="1419">
       <c r="A1419" t="n">
@@ -47445,6 +48588,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1421" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ilya.leontev</t>
+        </is>
+      </c>
     </row>
     <row r="1422">
       <c r="A1422" t="n">
@@ -47475,6 +48623,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1422" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kuhalsky</t>
+        </is>
+      </c>
     </row>
     <row r="1423">
       <c r="A1423" t="n">
@@ -47635,6 +48788,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1427" t="inlineStr">
+        <is>
+          <t>https://vk.ru/d.androsovtula</t>
+        </is>
+      </c>
     </row>
     <row r="1428">
       <c r="A1428" t="n">
@@ -47730,6 +48888,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1430" t="inlineStr">
+        <is>
+          <t>https://vk.ru/alexmarinkov</t>
+        </is>
+      </c>
     </row>
     <row r="1431">
       <c r="A1431" t="n">
@@ -47880,6 +49043,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1435" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sergeygrebenshchikov_tula</t>
+        </is>
+      </c>
     </row>
     <row r="1436">
       <c r="A1436" t="n">
@@ -47950,6 +49118,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1437" t="inlineStr">
+        <is>
+          <t>https://vk.ru/valentinsoin</t>
+        </is>
+      </c>
     </row>
     <row r="1438">
       <c r="A1438" t="n">
@@ -48020,6 +49193,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1439" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id626261588</t>
+        </is>
+      </c>
     </row>
     <row r="1440">
       <c r="A1440" t="n">
@@ -48050,6 +49228,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1440" t="inlineStr">
+        <is>
+          <t>https://vk.ru/novikov72rus</t>
+        </is>
+      </c>
     </row>
     <row r="1441">
       <c r="A1441" t="n">
@@ -48110,6 +49293,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1442" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sergey_morev72</t>
+        </is>
+      </c>
     </row>
     <row r="1443">
       <c r="A1443" t="n">
@@ -48245,6 +49433,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1446" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id156764092</t>
+        </is>
+      </c>
     </row>
     <row r="1447">
       <c r="A1447" t="n">
@@ -48275,6 +49468,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1447" t="inlineStr">
+        <is>
+          <t>https://vk.ru/za_zaytseva</t>
+        </is>
+      </c>
     </row>
     <row r="1448">
       <c r="A1448" t="n">
@@ -48335,6 +49533,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1449" t="inlineStr">
+        <is>
+          <t>https://vk.ru/apushkino2026</t>
+        </is>
+      </c>
     </row>
     <row r="1450">
       <c r="A1450" t="n">
@@ -48365,6 +49568,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1450" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id602119423</t>
+        </is>
+      </c>
     </row>
     <row r="1451">
       <c r="A1451" t="n">
@@ -48510,6 +49718,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1454" t="inlineStr">
+        <is>
+          <t>https://vk.ru/hvozdakivan</t>
+        </is>
+      </c>
     </row>
     <row r="1455">
       <c r="A1455" t="n">
@@ -48570,6 +49783,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1456" t="inlineStr">
+        <is>
+          <t>https://vk.ru/albert_usb</t>
+        </is>
+      </c>
     </row>
     <row r="1457">
       <c r="A1457" t="n">
@@ -48965,6 +50183,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1468" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id245420333</t>
+        </is>
+      </c>
     </row>
     <row r="1469">
       <c r="A1469" t="n">
@@ -49055,6 +50278,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1471" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kameko_vn</t>
+        </is>
+      </c>
     </row>
     <row r="1472">
       <c r="A1472" t="n">
@@ -49085,6 +50313,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1472" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id708130792</t>
+        </is>
+      </c>
     </row>
     <row r="1473">
       <c r="A1473" t="n">
@@ -49175,6 +50408,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1475" t="inlineStr">
+        <is>
+          <t>https://vk.ru/gradmitry</t>
+        </is>
+      </c>
     </row>
     <row r="1476">
       <c r="A1476" t="n">
@@ -49325,6 +50563,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1480" t="inlineStr">
+        <is>
+          <t>https://vk.ru/grigoriimatveev</t>
+        </is>
+      </c>
     </row>
     <row r="1481">
       <c r="A1481" t="n">
@@ -49385,6 +50628,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1482" t="inlineStr">
+        <is>
+          <t>https://vk.ru/roman_sultashov</t>
+        </is>
+      </c>
     </row>
     <row r="1483">
       <c r="A1483" t="n">
@@ -49510,6 +50758,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1486" t="inlineStr">
+        <is>
+          <t>https://vk.ru/m.aryapov</t>
+        </is>
+      </c>
     </row>
     <row r="1487">
       <c r="A1487" t="n">
@@ -49580,6 +50833,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1488" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kravchuk.official</t>
+        </is>
+      </c>
     </row>
     <row r="1489">
       <c r="A1489" t="n">
@@ -49790,6 +51048,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1495" t="inlineStr">
+        <is>
+          <t>https://vk.ru/i_ivanr</t>
+        </is>
+      </c>
     </row>
     <row r="1496">
       <c r="A1496" t="n">
@@ -50240,6 +51503,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1509" t="inlineStr">
+        <is>
+          <t>https://vk.ru/k.aidakov</t>
+        </is>
+      </c>
     </row>
     <row r="1510">
       <c r="A1510" t="n">
@@ -50270,6 +51538,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1510" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kornilov68</t>
+        </is>
+      </c>
     </row>
     <row r="1511">
       <c r="A1511" t="n">
@@ -50300,6 +51573,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1511" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id592278873</t>
+        </is>
+      </c>
     </row>
     <row r="1512">
       <c r="A1512" t="n">
@@ -50360,6 +51638,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1513" t="inlineStr">
+        <is>
+          <t>https://vk.ru/avsavintsev</t>
+        </is>
+      </c>
     </row>
     <row r="1514">
       <c r="A1514" t="n">
@@ -50390,6 +51673,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1514" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id6662430</t>
+        </is>
+      </c>
     </row>
     <row r="1515">
       <c r="A1515" t="n">
@@ -50450,6 +51738,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1516" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aksenov_da</t>
+        </is>
+      </c>
     </row>
     <row r="1517">
       <c r="A1517" t="n">
@@ -50510,6 +51803,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1518" t="inlineStr">
+        <is>
+          <t>https://vk.ru/edmitryk</t>
+        </is>
+      </c>
     </row>
     <row r="1519">
       <c r="A1519" t="n">
@@ -50630,6 +51928,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1522" t="inlineStr">
+        <is>
+          <t>https://vk.ru/vl_pashin</t>
+        </is>
+      </c>
     </row>
     <row r="1523">
       <c r="A1523" t="n">
@@ -50695,6 +51998,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1524" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ille174</t>
+        </is>
+      </c>
     </row>
     <row r="1525">
       <c r="A1525" t="n">
@@ -50815,6 +52123,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1528" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kurochkin__denis</t>
+        </is>
+      </c>
     </row>
     <row r="1529">
       <c r="A1529" t="n">
@@ -50875,6 +52188,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1530" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tural_novruzov</t>
+        </is>
+      </c>
     </row>
     <row r="1531">
       <c r="A1531" t="n">
@@ -50905,6 +52223,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1531" t="inlineStr">
+        <is>
+          <t>https://vk.ru/agkudinov</t>
+        </is>
+      </c>
     </row>
     <row r="1532">
       <c r="A1532" t="n">
@@ -50995,6 +52318,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1534" t="inlineStr">
+        <is>
+          <t>https://vk.ru/denisenko2026</t>
+        </is>
+      </c>
     </row>
     <row r="1535">
       <c r="A1535" t="n">
@@ -51025,6 +52353,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1535" t="inlineStr">
+        <is>
+          <t>https://vk.ru/egorbabkin24</t>
+        </is>
+      </c>
     </row>
     <row r="1536">
       <c r="A1536" t="n">
@@ -51055,6 +52388,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1536" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id10948205</t>
+        </is>
+      </c>
     </row>
     <row r="1537">
       <c r="A1537" t="n">
@@ -51145,6 +52483,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1539" t="inlineStr">
+        <is>
+          <t>https://vk.ru/polevapolina</t>
+        </is>
+      </c>
     </row>
     <row r="1540">
       <c r="A1540" t="n">
@@ -51240,6 +52583,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1542" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id291777428</t>
+        </is>
+      </c>
     </row>
     <row r="1543">
       <c r="A1543" t="n">
@@ -51270,6 +52618,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1543" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ryzhiyanton</t>
+        </is>
+      </c>
     </row>
     <row r="1544">
       <c r="A1544" t="n">
@@ -51330,6 +52683,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1545" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id471619851</t>
+        </is>
+      </c>
     </row>
     <row r="1546">
       <c r="A1546" t="n">
@@ -51450,6 +52808,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1549" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dremov.vladimir</t>
+        </is>
+      </c>
     </row>
     <row r="1550">
       <c r="A1550" t="n">
@@ -51480,6 +52843,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1550" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id264568069</t>
+        </is>
+      </c>
     </row>
     <row r="1551">
       <c r="A1551" t="n">
@@ -51510,6 +52878,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1551" t="inlineStr">
+        <is>
+          <t>https://vk.ru/besedin_a</t>
+        </is>
+      </c>
     </row>
     <row r="1552">
       <c r="A1552" t="n">
@@ -51540,6 +52913,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1552" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ar2r4ik</t>
+        </is>
+      </c>
     </row>
     <row r="1553">
       <c r="A1553" t="n">
@@ -51695,6 +53073,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1557" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sumind</t>
+        </is>
+      </c>
     </row>
     <row r="1558">
       <c r="A1558" t="n">
@@ -51725,6 +53108,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1558" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id296436217</t>
+        </is>
+      </c>
     </row>
     <row r="1559">
       <c r="A1559" t="n">
@@ -51975,6 +53363,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1566" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id817933153</t>
+        </is>
+      </c>
     </row>
     <row r="1567">
       <c r="A1567" t="n">
@@ -52007,7 +53400,7 @@
       </c>
       <c r="G1567" t="inlineStr">
         <is>
-          <t>https://vk.com/andreevkprf/</t>
+          <t>https://vk.com/andreevkprf/; https://vk.com/andreevkprf</t>
         </is>
       </c>
     </row>
@@ -52040,6 +53433,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1568" t="inlineStr">
+        <is>
+          <t>https://vk.ru/epetrov21</t>
+        </is>
+      </c>
     </row>
     <row r="1569">
       <c r="A1569" t="n">
@@ -52070,6 +53468,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1569" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1049035049</t>
+        </is>
+      </c>
     </row>
     <row r="1570">
       <c r="A1570" t="n">
@@ -52320,6 +53723,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1577" t="inlineStr">
+        <is>
+          <t>https://vk.ru/stepanovfm21</t>
+        </is>
+      </c>
     </row>
     <row r="1578">
       <c r="A1578" t="n">
@@ -52442,7 +53850,7 @@
       </c>
       <c r="G1581" t="inlineStr">
         <is>
-          <t>https://vk.com/konstantin_121; https://vk.com/club232057989</t>
+          <t>https://vk.com/konstantin_121;  https://vk.com/club232057989; https://vk.com/club232057989</t>
         </is>
       </c>
       <c r="H1581" t="inlineStr">
@@ -52487,7 +53895,7 @@
       </c>
       <c r="G1582" t="inlineStr">
         <is>
-          <t>http://vk.com/id656175910; https://vk.com/id656175910</t>
+          <t>http://vk.com/id656175910;  https://vk.com/id656175910; https://vk.com/id656175910</t>
         </is>
       </c>
       <c r="H1582" t="inlineStr">
@@ -52620,6 +54028,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1586" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dudorovan</t>
+        </is>
+      </c>
     </row>
     <row r="1587">
       <c r="A1587" t="n">
@@ -52680,6 +54093,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1588" t="inlineStr">
+        <is>
+          <t>https://vk.ru/faberlic87</t>
+        </is>
+      </c>
     </row>
     <row r="1589">
       <c r="A1589" t="n">
@@ -52815,6 +54233,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1592" t="inlineStr">
+        <is>
+          <t>https://vk.ru/lamdo1990</t>
+        </is>
+      </c>
     </row>
     <row r="1593">
       <c r="A1593" t="n">
@@ -52935,6 +54358,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1596" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id44807596</t>
+        </is>
+      </c>
     </row>
     <row r="1597">
       <c r="A1597" t="n">
@@ -53055,6 +54483,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1600" t="inlineStr">
+        <is>
+          <t>https://vk.ru/deputatkuznetsowa</t>
+        </is>
+      </c>
     </row>
     <row r="1601">
       <c r="A1601" t="n">
@@ -53120,6 +54553,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1602" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id32251143</t>
+        </is>
+      </c>
     </row>
     <row r="1603">
       <c r="A1603" t="n">
@@ -53310,6 +54748,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1608" t="inlineStr">
+        <is>
+          <t>https://vk.ru/molchanovartem76</t>
+        </is>
+      </c>
     </row>
     <row r="1609">
       <c r="A1609" t="n">
@@ -53380,6 +54823,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1610" t="inlineStr">
+        <is>
+          <t>https://vk.ru/gorokhov087</t>
+        </is>
+      </c>
     </row>
     <row r="1611">
       <c r="A1611" t="n">
@@ -53408,6 +54856,43 @@
       <c r="F1611" t="inlineStr">
         <is>
           <t>ЛДПР</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>Самарская область</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>Округ № 160 (Тольяттинский)</t>
+        </is>
+      </c>
+      <c r="D1612" t="inlineStr">
+        <is>
+          <t>Округ включает Центральный и Автозаводский районы города Тольятти, а также основную часть пригородного Ставропольского района.</t>
+        </is>
+      </c>
+      <c r="E1612" t="inlineStr">
+        <is>
+          <t>Мотрюков Владимир Анатольевич</t>
+        </is>
+      </c>
+      <c r="F1612" t="inlineStr">
+        <is>
+          <t>Новые люди</t>
+        </is>
+      </c>
+      <c r="G1612" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id75270050</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: merge green-only VK accounts from found-but-not-added sheet
</commit_message>
<xml_diff>
--- a/candidates.xlsx
+++ b/candidates.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="17970" windowHeight="8100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Кандидаты по округам" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Кандидаты по округам" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -1338,6 +1338,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://vk.com/id163661797</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3178,6 +3183,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://vk.com/public79363208</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3828,6 +3838,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id825825456</t>
+        </is>
+      </c>
       <c r="H100" t="inlineStr">
         <is>
           <t>t.me/GrafinyaNegoduet</t>
@@ -4158,6 +4173,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id200001986892</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4943,6 +4963,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1107838890</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -7008,6 +7033,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id662804207</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -9393,6 +9423,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>https://vk.ru/chaika_officiaal; https://vk.ru/id785219714</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -10488,6 +10523,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>https://vk.ru/andrey_iglin</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -11048,6 +11088,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>https://vk.com/public232909640</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -14315,7 +14360,7 @@
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t>https://vk.com/aleksandr_iltakov</t>
+          <t>https://vk.com/aleksandr_iltakov; https://vk.ru/a.iltyakov</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
@@ -15653,6 +15698,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>https://vk.com/public233972571</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="n">
@@ -16413,6 +16463,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>https://vk.com/public240381657</t>
+        </is>
+      </c>
     </row>
     <row r="478">
       <c r="A478" t="n">
@@ -18958,6 +19013,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>https://vk.com/public214208838</t>
+        </is>
+      </c>
       <c r="H544" t="inlineStr">
         <is>
           <t>https://t.me/ivanov_moto</t>
@@ -21708,6 +21768,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>https://vk.ru/yurovsg</t>
+        </is>
+      </c>
     </row>
     <row r="617">
       <c r="A617" t="n">
@@ -22498,6 +22563,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>https://vk.ru/nikolai_shcherbak</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" t="n">
@@ -22560,7 +22630,7 @@
       </c>
       <c r="G642" t="inlineStr">
         <is>
-          <t>https://vk.com/kolunov_s</t>
+          <t>https://vk.com/kolunov_s; https://vk.com/sergey.kolunov; https://vk.ru/kolunov_s</t>
         </is>
       </c>
       <c r="H642" t="inlineStr">
@@ -23228,6 +23298,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>https://vk.ru/club232220187</t>
+        </is>
+      </c>
     </row>
     <row r="663">
       <c r="A663" t="n">
@@ -23603,6 +23678,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id52065716</t>
+        </is>
+      </c>
     </row>
     <row r="674">
       <c r="A674" t="n">
@@ -23858,6 +23938,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ger77rus</t>
+        </is>
+      </c>
     </row>
     <row r="682">
       <c r="A682" t="n">
@@ -24018,6 +24103,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>https://vk.com/perepelkin_sv; https://vk.ru/d06rwi</t>
+        </is>
+      </c>
     </row>
     <row r="687">
       <c r="A687" t="n">
@@ -28228,6 +28318,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>https://vk.ru/deputat_bondarenko_andrey</t>
+        </is>
+      </c>
     </row>
     <row r="813">
       <c r="A813" t="n">
@@ -29158,6 +29253,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>https://vk.ru/raschupkin1987</t>
+        </is>
+      </c>
     </row>
     <row r="840">
       <c r="A840" t="n">
@@ -31133,6 +31233,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id148207959</t>
+        </is>
+      </c>
     </row>
     <row r="898">
       <c r="A898" t="n">
@@ -31308,6 +31413,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id437409472</t>
+        </is>
+      </c>
     </row>
     <row r="903">
       <c r="A903" t="n">
@@ -31338,6 +31448,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>https://vk.ru/club240452336</t>
+        </is>
+      </c>
     </row>
     <row r="904">
       <c r="A904" t="n">
@@ -31368,6 +31483,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>https://vk.ru/motivationapakaev</t>
+        </is>
+      </c>
     </row>
     <row r="905">
       <c r="A905" t="n">
@@ -31463,6 +31583,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>https://vk.ru/p.railko</t>
+        </is>
+      </c>
     </row>
     <row r="908">
       <c r="A908" t="n">
@@ -32088,6 +32213,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>https://vk.com/sradygea</t>
+        </is>
+      </c>
     </row>
     <row r="927">
       <c r="A927" t="n">
@@ -32118,6 +32248,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>https://vk.ru/tembotshovgenov</t>
+        </is>
+      </c>
     </row>
     <row r="928">
       <c r="A928" t="n">
@@ -32373,6 +32508,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>https://vk.com/public195422568; https://vk.ru/id1066720687</t>
+        </is>
+      </c>
     </row>
     <row r="936">
       <c r="A936" t="n">
@@ -32833,6 +32973,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>https://vk.ru/laisan_ka</t>
+        </is>
+      </c>
     </row>
     <row r="950">
       <c r="A950" t="n">
@@ -34068,6 +34213,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>https://vk.ru/shirip87</t>
+        </is>
+      </c>
     </row>
     <row r="987">
       <c r="A987" t="n">
@@ -34558,6 +34708,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id1109251149</t>
+        </is>
+      </c>
     </row>
     <row r="1002">
       <c r="A1002" t="n">
@@ -34953,6 +35108,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>https://vk.ru/frantsuzov08</t>
+        </is>
+      </c>
     </row>
     <row r="1014">
       <c r="A1014" t="n">
@@ -35308,6 +35468,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1024" t="inlineStr">
+        <is>
+          <t>https://vk.ru/chagen</t>
+        </is>
+      </c>
     </row>
     <row r="1025">
       <c r="A1025" t="n">
@@ -35803,6 +35968,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id828698969</t>
+        </is>
+      </c>
     </row>
     <row r="1040">
       <c r="A1040" t="n">
@@ -36153,6 +36323,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1050" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id489269664</t>
+        </is>
+      </c>
     </row>
     <row r="1051">
       <c r="A1051" t="n">
@@ -36308,6 +36483,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1055" t="inlineStr">
+        <is>
+          <t>https://vk.ru/uhroman</t>
+        </is>
+      </c>
     </row>
     <row r="1056">
       <c r="A1056" t="n">
@@ -36728,6 +36908,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sher100bitov</t>
+        </is>
+      </c>
     </row>
     <row r="1068">
       <c r="A1068" t="n">
@@ -37188,6 +37373,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>https://vk.ru/petr_shamaev</t>
+        </is>
+      </c>
     </row>
     <row r="1082">
       <c r="A1082" t="n">
@@ -37588,6 +37778,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id16049337</t>
+        </is>
+      </c>
     </row>
     <row r="1094">
       <c r="A1094" t="n">
@@ -37648,6 +37843,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>https://vk.ru/d.chirkov76</t>
+        </is>
+      </c>
     </row>
     <row r="1096">
       <c r="A1096" t="n">
@@ -38363,6 +38563,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>https://vk.ru/marsel_shaydullin</t>
+        </is>
+      </c>
     </row>
     <row r="1117">
       <c r="A1117" t="n">
@@ -38493,6 +38698,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dinara_khalimdarova</t>
+        </is>
+      </c>
     </row>
     <row r="1121">
       <c r="A1121" t="n">
@@ -38558,6 +38768,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>https://vk.ru/sovetnik116</t>
+        </is>
+      </c>
     </row>
     <row r="1123">
       <c r="A1123" t="n">
@@ -38763,6 +38978,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aidysmaachadamba9494</t>
+        </is>
+      </c>
     </row>
     <row r="1129">
       <c r="A1129" t="n">
@@ -39038,6 +39258,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id200000565243</t>
+        </is>
+      </c>
     </row>
     <row r="1137">
       <c r="A1137" t="n">
@@ -39133,6 +39358,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>https://vk.ru/llavr</t>
+        </is>
+      </c>
     </row>
     <row r="1140">
       <c r="A1140" t="n">
@@ -39163,6 +39393,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>https://vk.ru/chukhlebovalex; https://vk.ru/id100075866</t>
+        </is>
+      </c>
     </row>
     <row r="1141">
       <c r="A1141" t="n">
@@ -39523,6 +39758,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>https://vk.ru/fruit007; https://vk.ru/maxfedorov75</t>
+        </is>
+      </c>
     </row>
     <row r="1152">
       <c r="A1152" t="n">
@@ -40098,6 +40338,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>https://vk.ru/general_huade</t>
+        </is>
+      </c>
     </row>
     <row r="1169">
       <c r="A1169" t="n">
@@ -40343,6 +40588,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dinfatina</t>
+        </is>
+      </c>
     </row>
     <row r="1176">
       <c r="A1176" t="n">
@@ -40518,6 +40768,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id105467973</t>
+        </is>
+      </c>
     </row>
     <row r="1181">
       <c r="A1181" t="n">
@@ -40883,6 +41138,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1191" t="inlineStr">
+        <is>
+          <t>https://vk.ru/a.fetisov63</t>
+        </is>
+      </c>
     </row>
     <row r="1192">
       <c r="A1192" t="n">
@@ -42503,6 +42763,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1239" t="inlineStr">
+        <is>
+          <t>https://vk.ru/square_hammer</t>
+        </is>
+      </c>
     </row>
     <row r="1240">
       <c r="A1240" t="n">
@@ -42763,6 +43028,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1247" t="inlineStr">
+        <is>
+          <t>https://vk.ru/club240836290</t>
+        </is>
+      </c>
     </row>
     <row r="1248">
       <c r="A1248" t="n">
@@ -42888,6 +43158,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1251" t="inlineStr">
+        <is>
+          <t>https://vk.ru/aleksandr.ustimenko</t>
+        </is>
+      </c>
     </row>
     <row r="1252">
       <c r="A1252" t="n">
@@ -42948,6 +43223,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1253" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ishmakov71</t>
+        </is>
+      </c>
     </row>
     <row r="1254">
       <c r="A1254" t="n">
@@ -43490,7 +43770,7 @@
       </c>
       <c r="G1269" t="inlineStr">
         <is>
-          <t>https://vk.com/milonov</t>
+          <t>https://vk.com/milonov; https://vk.com/vvmilonov; https://vk.ru/milonov</t>
         </is>
       </c>
       <c r="H1269" t="inlineStr">
@@ -43958,6 +44238,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1283" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ilyaballet; https://vk.ru/kuznetsovil</t>
+        </is>
+      </c>
     </row>
     <row r="1284">
       <c r="A1284" t="n">
@@ -44183,6 +44468,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>https://vk.ru/hatsenko</t>
+        </is>
+      </c>
     </row>
     <row r="1291">
       <c r="A1291" t="n">
@@ -44473,6 +44763,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>https://vk.ru/alexandr_janklovich</t>
+        </is>
+      </c>
     </row>
     <row r="1300">
       <c r="A1300" t="n">
@@ -44918,6 +45213,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>https://vk.ru/m.chiryshev</t>
+        </is>
+      </c>
     </row>
     <row r="1313">
       <c r="A1313" t="n">
@@ -45713,6 +46013,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id67126166</t>
+        </is>
+      </c>
     </row>
     <row r="1336">
       <c r="A1336" t="n">
@@ -46353,6 +46658,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>https://vk.ru/chudov1</t>
+        </is>
+      </c>
     </row>
     <row r="1355">
       <c r="A1355" t="n">
@@ -46673,6 +46983,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1363" t="inlineStr">
+        <is>
+          <t>https://vk.ru/club212502738</t>
+        </is>
+      </c>
     </row>
     <row r="1364">
       <c r="A1364" t="n">
@@ -47093,6 +47408,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>https://vk.ru/shuvaev_di</t>
+        </is>
+      </c>
     </row>
     <row r="1377">
       <c r="A1377" t="n">
@@ -47123,6 +47443,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id327186917</t>
+        </is>
+      </c>
     </row>
     <row r="1378">
       <c r="A1378" t="n">
@@ -47433,6 +47758,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id393714186</t>
+        </is>
+      </c>
     </row>
     <row r="1388">
       <c r="A1388" t="n">
@@ -48658,6 +48988,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1423" t="inlineStr">
+        <is>
+          <t>https://vk.ru/valodarm</t>
+        </is>
+      </c>
     </row>
     <row r="1424">
       <c r="A1424" t="n">
@@ -48823,6 +49158,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1428" t="inlineStr">
+        <is>
+          <t>https://vk.ru/yuribrovko</t>
+        </is>
+      </c>
     </row>
     <row r="1429">
       <c r="A1429" t="n">
@@ -48923,6 +49263,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1431" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id712412021</t>
+        </is>
+      </c>
     </row>
     <row r="1432">
       <c r="A1432" t="n">
@@ -49328,6 +49673,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1443" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ivan_ldpr</t>
+        </is>
+      </c>
     </row>
     <row r="1444">
       <c r="A1444" t="n">
@@ -50048,6 +50398,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1464" t="inlineStr">
+        <is>
+          <t>https://vk.ru/ssstasssik</t>
+        </is>
+      </c>
     </row>
     <row r="1465">
       <c r="A1465" t="n">
@@ -50248,6 +50603,11 @@
           <t>Новые люди</t>
         </is>
       </c>
+      <c r="G1470" t="inlineStr">
+        <is>
+          <t>https://vk.ru/yurabel0usov</t>
+        </is>
+      </c>
     </row>
     <row r="1471">
       <c r="A1471" t="n">
@@ -50868,6 +51228,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1489" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id780503556</t>
+        </is>
+      </c>
     </row>
     <row r="1490">
       <c r="A1490" t="n">
@@ -51143,6 +51508,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1498" t="inlineStr">
+        <is>
+          <t>https://vk.ru/batyu_ruslan</t>
+        </is>
+      </c>
     </row>
     <row r="1499">
       <c r="A1499" t="n">
@@ -51608,6 +51978,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1512" t="inlineStr">
+        <is>
+          <t>https://vk.ru/alexeyanosov</t>
+        </is>
+      </c>
     </row>
     <row r="1513">
       <c r="A1513" t="n">
@@ -52158,6 +52533,11 @@
           <t>Справедливая Россия</t>
         </is>
       </c>
+      <c r="G1529" t="inlineStr">
+        <is>
+          <t>https://vk.ru/shvetsov_vasiliy</t>
+        </is>
+      </c>
     </row>
     <row r="1530">
       <c r="A1530" t="n">
@@ -52748,6 +53128,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1547" t="inlineStr">
+        <is>
+          <t>https://vk.ru/katherinedirector</t>
+        </is>
+      </c>
     </row>
     <row r="1548">
       <c r="A1548" t="n">
@@ -53143,6 +53528,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1559" t="inlineStr">
+        <is>
+          <t>https://vk.ru/valentin1917</t>
+        </is>
+      </c>
     </row>
     <row r="1560">
       <c r="A1560" t="n">
@@ -53203,6 +53593,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1561" t="inlineStr">
+        <is>
+          <t>https://vk.ru/kozhevnikov_km</t>
+        </is>
+      </c>
     </row>
     <row r="1562">
       <c r="A1562" t="n">
@@ -53233,6 +53628,11 @@
           <t>ЛДПР</t>
         </is>
       </c>
+      <c r="G1562" t="inlineStr">
+        <is>
+          <t>https://vk.ru/dj_umarov; https://vk.ru/ldpr_95</t>
+        </is>
+      </c>
     </row>
     <row r="1563">
       <c r="A1563" t="n">
@@ -53593,6 +53993,11 @@
           <t>Единая Россия</t>
         </is>
       </c>
+      <c r="G1573" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id438613823</t>
+        </is>
+      </c>
     </row>
     <row r="1574">
       <c r="A1574" t="n">
@@ -53758,6 +54163,11 @@
           <t>КПРФ</t>
         </is>
       </c>
+      <c r="G1578" t="inlineStr">
+        <is>
+          <t>https://vk.ru/chuvashiasila21</t>
+        </is>
+      </c>
     </row>
     <row r="1579">
       <c r="A1579" t="n">
@@ -54856,6 +55266,11 @@
       <c r="F1611" t="inlineStr">
         <is>
           <t>ЛДПР</t>
+        </is>
+      </c>
+      <c r="G1611" t="inlineStr">
+        <is>
+          <t>https://vk.ru/id806532652</t>
         </is>
       </c>
     </row>

</xml_diff>